<commit_message>
feat: Implement a payroll report dashboard with earnings, deductions, and department summaries, and add attendance timecard functionality.
</commit_message>
<xml_diff>
--- a/thaco/Thaco Project Kick off Sheet (1).xlsx
+++ b/thaco/Thaco Project Kick off Sheet (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/gitlocal/thaco/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9162D3B-3AED-0143-AEE7-BC577AC76B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99184871-2520-7D40-BAA9-124C620DBA3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="34440" windowHeight="20040" activeTab="4" xr2:uid="{974542BB-E32D-A94E-A51C-E9B15B50DB02}"/>
+    <workbookView xWindow="40780" yWindow="820" windowWidth="30820" windowHeight="20060" activeTab="4" xr2:uid="{974542BB-E32D-A94E-A51C-E9B15B50DB02}"/>
   </bookViews>
   <sheets>
     <sheet name="Meeting Summary" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
     <sheet name="Approval Matrix" sheetId="6" r:id="rId7"/>
     <sheet name="Templates Requirments" sheetId="8" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="296">
   <si>
     <t>Giai đoạn /Phase</t>
   </si>
@@ -2012,6 +2012,21 @@
   </si>
   <si>
     <t>4 weeks</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Not started</t>
   </si>
 </sst>
 </file>
@@ -2116,7 +2131,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2192,6 +2207,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2313,7 +2346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2383,6 +2416,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2405,13 +2445,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>17</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>101600</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>381000</xdr:rowOff>
@@ -2775,352 +2815,434 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C64EBA2-0CB3-A94A-AFCB-6E2F4E8E07D8}">
-  <dimension ref="A1:AA27"/>
+  <dimension ref="A1:AB27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="23" width="2.83203125" customWidth="1"/>
-    <col min="24" max="28" width="3" customWidth="1"/>
-    <col min="29" max="33" width="3.33203125" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="49.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="24" width="2.83203125" customWidth="1"/>
+    <col min="25" max="29" width="3" customWidth="1"/>
+    <col min="30" max="34" width="3.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
         <v>247</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="D1" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="E1" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="E1" s="27"/>
       <c r="F1" s="27"/>
       <c r="G1" s="27"/>
       <c r="H1" s="27"/>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="27"/>
+      <c r="J1" s="28" t="s">
         <v>251</v>
       </c>
-      <c r="J1" s="28"/>
       <c r="K1" s="28"/>
       <c r="L1" s="28"/>
       <c r="M1" s="28"/>
-      <c r="N1" s="29" t="s">
+      <c r="N1" s="28"/>
+      <c r="O1" s="29" t="s">
         <v>252</v>
       </c>
-      <c r="O1" s="29"/>
       <c r="P1" s="29"/>
       <c r="Q1" s="29"/>
       <c r="R1" s="29"/>
-      <c r="S1" s="30" t="s">
+      <c r="S1" s="29"/>
+      <c r="T1" s="30" t="s">
         <v>253</v>
       </c>
-      <c r="T1" s="30"/>
       <c r="U1" s="30"/>
       <c r="V1" s="30"/>
       <c r="W1" s="30"/>
-    </row>
-    <row r="2" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="X1" s="30"/>
+    </row>
+    <row r="2" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" s="37" t="s">
         <v>255</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="D2" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="D2" s="22"/>
-    </row>
-    <row r="3" spans="1:23" ht="40" x14ac:dyDescent="0.25">
+      <c r="E2" s="22"/>
+    </row>
+    <row r="3" spans="1:24" ht="40" x14ac:dyDescent="0.25">
       <c r="A3" s="20"/>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="35" t="s">
+        <v>292</v>
+      </c>
+      <c r="C3" s="37" t="s">
         <v>257</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="D3" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="E3" s="22"/>
-    </row>
-    <row r="4" spans="1:23" ht="40" x14ac:dyDescent="0.25">
+      <c r="F3" s="22"/>
+    </row>
+    <row r="4" spans="1:24" ht="40" x14ac:dyDescent="0.25">
       <c r="A4" s="20"/>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C4" s="37" t="s">
         <v>259</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="D4" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="E4" s="22"/>
-    </row>
-    <row r="5" spans="1:23" ht="40" x14ac:dyDescent="0.25">
+      <c r="F4" s="22"/>
+    </row>
+    <row r="5" spans="1:24" ht="40" x14ac:dyDescent="0.25">
       <c r="A5" s="20"/>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C5" s="37" t="s">
         <v>260</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="D5" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="E5" s="22"/>
-    </row>
-    <row r="6" spans="1:23" ht="40" x14ac:dyDescent="0.25">
+      <c r="F5" s="22"/>
+    </row>
+    <row r="6" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A6" s="20"/>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C6" s="38" t="s">
         <v>261</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="D6" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="F6" s="22"/>
+    </row>
+    <row r="7" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A7" s="20"/>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="39" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="37" t="s">
         <v>262</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="D7" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="F7" s="22"/>
-    </row>
-    <row r="8" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="G7" s="22"/>
+    </row>
+    <row r="8" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A8" s="20"/>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="37" t="s">
         <v>263</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="D8" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="F8" s="22"/>
-    </row>
-    <row r="9" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="G8" s="22"/>
+    </row>
+    <row r="9" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A9" s="20"/>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C9" s="37" t="s">
         <v>264</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="D9" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="F9" s="22"/>
-    </row>
-    <row r="10" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="G9" s="22"/>
+    </row>
+    <row r="10" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A10" s="20"/>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C10" s="37" t="s">
         <v>265</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="D10" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="G10" s="22"/>
       <c r="H10" s="22"/>
-    </row>
-    <row r="11" spans="1:23" ht="40" x14ac:dyDescent="0.25">
+      <c r="I10" s="22"/>
+    </row>
+    <row r="11" spans="1:24" ht="40" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="39" t="s">
+        <v>294</v>
+      </c>
+      <c r="C11" s="37" t="s">
         <v>267</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="D11" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="D11" s="23"/>
-    </row>
-    <row r="12" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="E11" s="23"/>
+    </row>
+    <row r="12" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A12" s="20"/>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="37" t="s">
         <v>268</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="D12" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="E12" s="23"/>
-    </row>
-    <row r="13" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="F12" s="23"/>
+    </row>
+    <row r="13" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A13" s="20"/>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="39" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="37" t="s">
         <v>269</v>
       </c>
-      <c r="C13" s="21" t="s">
+      <c r="D13" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="E13" s="23"/>
-    </row>
-    <row r="14" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="F13" s="23"/>
+    </row>
+    <row r="14" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A14" s="20"/>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="36" t="s">
+        <v>293</v>
+      </c>
+      <c r="C14" s="38" t="s">
         <v>270</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="D14" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="F14" s="23"/>
       <c r="G14" s="23"/>
       <c r="H14" s="23"/>
-    </row>
-    <row r="15" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="I14" s="23"/>
+    </row>
+    <row r="15" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C15" s="21" t="s">
         <v>273</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="D15" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="D15" s="24"/>
       <c r="E15" s="24"/>
-    </row>
-    <row r="16" spans="1:23" ht="20" x14ac:dyDescent="0.25">
+      <c r="F15" s="24"/>
+    </row>
+    <row r="16" spans="1:24" ht="20" x14ac:dyDescent="0.25">
       <c r="A16" s="20"/>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="D16" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="F16" s="24"/>
-    </row>
-    <row r="17" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="G16" s="24"/>
+    </row>
+    <row r="17" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A17" s="20"/>
-      <c r="B17" s="21" t="s">
+      <c r="B17" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>276</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="F17" s="24"/>
-    </row>
-    <row r="18" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A18" s="20"/>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="D18" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="F18" s="24"/>
-    </row>
-    <row r="19" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A19" s="20"/>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C19" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="D19" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="G19" s="24"/>
-    </row>
-    <row r="20" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="H19" s="24"/>
+    </row>
+    <row r="20" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A20" s="20"/>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C20" s="21" t="s">
         <v>279</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="D20" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="H20" s="24"/>
-    </row>
-    <row r="21" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="I20" s="24"/>
+    </row>
+    <row r="21" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A21" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="D21" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="I21" s="25"/>
       <c r="J21" s="25"/>
-    </row>
-    <row r="22" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="K21" s="25"/>
+    </row>
+    <row r="22" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A22" s="20"/>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="D22" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="K22" s="25"/>
       <c r="L22" s="25"/>
       <c r="M22" s="25"/>
       <c r="N22" s="25"/>
       <c r="O22" s="25"/>
       <c r="P22" s="25"/>
-    </row>
-    <row r="23" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="Q22" s="25"/>
+    </row>
+    <row r="23" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A23" s="20"/>
-      <c r="B23" s="21" t="s">
+      <c r="B23" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>283</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="D23" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="Q23" s="25"/>
       <c r="R23" s="25"/>
-    </row>
-    <row r="24" spans="1:27" ht="40" x14ac:dyDescent="0.25">
+      <c r="S23" s="25"/>
+    </row>
+    <row r="24" spans="1:28" ht="40" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>285</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="D24" s="21" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="25" spans="1:27" ht="40" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" ht="40" x14ac:dyDescent="0.25">
       <c r="A25" s="20"/>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C25" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="D25" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="S25" s="26"/>
       <c r="T25" s="26"/>
-    </row>
-    <row r="26" spans="1:27" ht="40" x14ac:dyDescent="0.25">
+      <c r="U25" s="26"/>
+    </row>
+    <row r="26" spans="1:28" ht="40" x14ac:dyDescent="0.25">
       <c r="A26" s="20"/>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>287</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="D26" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="U26" s="26"/>
       <c r="V26" s="26"/>
       <c r="W26" s="26"/>
-    </row>
-    <row r="27" spans="1:27" ht="20" x14ac:dyDescent="0.25">
+      <c r="X26" s="26"/>
+    </row>
+    <row r="27" spans="1:28" ht="20" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="20" t="s">
+        <v>295</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>289</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="D27" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="X27" s="22"/>
-      <c r="Y27" s="22" t="s">
+      <c r="Y27" s="22"/>
+      <c r="Z27" s="22" t="s">
         <v>290</v>
       </c>
-      <c r="Z27" s="22"/>
       <c r="AA27" s="22"/>
+      <c r="AB27" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="D1:H1"/>
-    <mergeCell ref="I1:M1"/>
-    <mergeCell ref="N1:R1"/>
-    <mergeCell ref="S1:W1"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="J1:N1"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="T1:X1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>